<commit_message>
Rewrite the remaining syllabi and add planned figures
All disciplines except UIFIS, MAPO and project management now have real chapter summaries, measurable outcomes and topic lists instead of placeholder text. The plans carry 88 planned figures, and the certification plan gained 12 inline diagrams that are also present in its lectures.
</commit_message>
<xml_diff>
--- a/courses/2/algorithms/dist/Учебный_план_Основы_алгоритмизации_и_программирования.xlsx
+++ b/courses/2/algorithms/dist/Учебный_план_Основы_алгоритмизации_и_программирования.xlsx
@@ -174,7 +174,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="45" customHeight="1">
+    <row r="6" ht="60" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
@@ -195,12 +195,12 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Разбор темы «Алгоритм и его свойства»: ключевые понятия, примеры и практические ситуации.</t>
+          <t xml:space="preserve">Разберёте, чем алгоритм отличается от любой последовательности действий, и научитесь проверять запись на дискретность, конечность и результативность.</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Алгоритм и его свойства</t>
+          <t xml:space="preserve">исполнитель, дискретность, детерминированность, конечность, массовость</t>
         </is>
       </c>
     </row>
@@ -225,12 +225,12 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Разбор темы «Блок-схемы и псевдокод»: ключевые понятия, примеры и практические ситуации.</t>
+          <t xml:space="preserve">Научитесь переводить словесное описание в блок-схему по ГОСТ и в псевдокод, чтобы один и тот же алгоритм читался двумя способами.</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Блок-схемы и псевдокод</t>
+          <t xml:space="preserve">терминатор, процесс, решение, соединитель, стрелка перехода</t>
         </is>
       </c>
     </row>
@@ -255,12 +255,12 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Совмещённая практическая работа: Ввод и вывод: базовые задачи; Арифметические операции: базовые задачи.</t>
+          <t xml:space="preserve">Пишете в VS Code программы, которые читают числа через input и печатают результат арифметики, и сдаёте набор из пяти работающих скриптов с выводом.</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ввод и вывод: базовые задачи, Арифметические операции: базовые задачи</t>
+          <t xml:space="preserve">input, int, float, f-строка, деление нацело, остаток</t>
         </is>
       </c>
     </row>
@@ -285,12 +285,12 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Разбор темы «Переменные, типы и выражения»: ключевые понятия, примеры и практические ситуации.</t>
+          <t xml:space="preserve">Разберёте, как Python хранит значение в переменной, почему 0.1 + 0.2 даёт хвост и когда неявное приведение типов ломает расчёт.</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Переменные, типы и выражения</t>
+          <t xml:space="preserve">переменная, динамическая типизация, приведение типов, приоритет операций, округление</t>
         </is>
       </c>
     </row>
@@ -315,12 +315,12 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Разбор темы «Условия и выбор»: ключевые понятия, примеры и практические ситуации.</t>
+          <t xml:space="preserve">Научитесь строить ветвление на if, elif и else и выбирать между лестницей условий и словарём вариантов, когда ветвей становится много.</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Условия и выбор</t>
+          <t xml:space="preserve">if, elif, else, логические операторы, граничный случай</t>
         </is>
       </c>
     </row>
@@ -345,16 +345,16 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Совмещённая практическая работа: Разветвления: базовые задачи; Циклы for: базовые задачи.</t>
+          <t xml:space="preserve">Решаете задачи на выбор варианта и перебор диапазона: программы с if, elif и for, проверенные на наборе входных значений.</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Разветвления: базовые задачи, Циклы for: базовые задачи</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="30" customHeight="1">
+          <t xml:space="preserve">range, ветвление, счётчик, накопление суммы, тестовый набор</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="45" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">9</t>
@@ -375,12 +375,12 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Разбор темы «Циклы»: ключевые понятия, примеры и практические ситуации.</t>
+          <t xml:space="preserve">Сравните for и while, разберёте, откуда берётся бесконечный цикл, и научитесь останавливать перебор через break и continue.</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Циклы</t>
+          <t xml:space="preserve">for, while, break, continue, счётчик итераций, условие выхода</t>
         </is>
       </c>
     </row>
@@ -405,12 +405,12 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Разбор темы «Массивы и списки»: ключевые понятия, примеры и практические ситуации.</t>
+          <t xml:space="preserve">Разберёте, как список хранит элементы по индексам, что делает срез и почему вставка в середину дороже добавления в конец.</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Массивы и списки</t>
+          <t xml:space="preserve">индекс, срез, append, вложенный список, длина списка</t>
         </is>
       </c>
     </row>
@@ -435,16 +435,16 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Совмещённая практическая работа: Циклы while: базовые задачи; Вложенные циклы: базовые задачи.</t>
+          <t xml:space="preserve">Пишете программы с while и вложенным перебором: таблицы, суммы рядов и поиск до условия, с проверкой числа итераций.</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Циклы while: базовые задачи, Вложенные циклы: базовые задачи</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1">
+          <t xml:space="preserve">while True, вложенный цикл, внешний счётчик, таблица, валидация ввода</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="45" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">13</t>
@@ -465,12 +465,12 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Разбор темы «Строки»: ключевые понятия, примеры и практические ситуации.</t>
+          <t xml:space="preserve">Научитесь резать строку по индексам, собирать её из частей и разбирать текст на слова без регулярных выражений.</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Строки</t>
+          <t xml:space="preserve">неизменяемость, split, join, strip, юникод, форматирование</t>
         </is>
       </c>
     </row>
@@ -495,12 +495,12 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Разбор темы «Функции и модули»: ключевые понятия, примеры и практические ситуации.</t>
+          <t xml:space="preserve">Разберёте, зачем выносить код в функцию, как передаются аргументы и как собрать свои функции в модуль, который импортируют другие файлы.</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Функции и модули</t>
+          <t xml:space="preserve">def, return, параметр, область видимости, import, докстрока</t>
         </is>
       </c>
     </row>
@@ -525,12 +525,12 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Совмещённая практическая работа: Строки: базовые задачи; Списки: базовые задачи.</t>
+          <t xml:space="preserve">Обрабатываете текст и наборы данных: подсчёт слов, очистка строк, сортировка списка, и сдаёте скрипты с разбором сложных случаев.</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Строки: базовые задачи, Списки: базовые задачи</t>
+          <t xml:space="preserve">частота, фильтрация, сортировка, пустой ввод, нормализация</t>
         </is>
       </c>
     </row>
@@ -555,12 +555,12 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Разбор темы «Словари и множества»: ключевые понятия, примеры и практические ситуации.</t>
+          <t xml:space="preserve">Разберёте, как словарь находит значение по ключу за один шаг, чем множество отличается от списка и где теряется порядок элементов.</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Словари и множества</t>
+          <t xml:space="preserve">ключ, значение, хеш, set, уникальность, перебор items</t>
         </is>
       </c>
     </row>
@@ -585,12 +585,12 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Разбор темы «Файлы и обработка данных»: ключевые понятия, примеры и практические ситуации.</t>
+          <t xml:space="preserve">Научитесь читать и записывать текстовые файлы через with, не теряя данные при ошибке, и обрабатывать строки файла построчно.</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Файлы и обработка данных</t>
+          <t xml:space="preserve">open, with, режим доступа, кодировка, чтение строк, буфер</t>
         </is>
       </c>
     </row>
@@ -615,12 +615,12 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Совмещённая практическая работа: Кортежи: базовые задачи; Словари: базовые задачи.</t>
+          <t xml:space="preserve">Работаете с неизменяемыми наборами и справочниками: кортеж как ключ, словарь как база записей, и сдаёте программу с отчётом по данным.</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Кортежи: базовые задачи, Словари: базовые задачи</t>
+          <t xml:space="preserve">неизменяемый набор, распаковка, вложенный словарь, get, обновление записи</t>
         </is>
       </c>
     </row>
@@ -645,16 +645,16 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Разбор темы «Ошибки, исключения и отладка»: ключевые понятия, примеры и практические ситуации.</t>
+          <t xml:space="preserve">Разберёте три вида ошибок, научитесь читать трассировку Python и обрабатывать сбой через try, except и finally вместо падения программы.</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ошибки, исключения и отладка</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="45" customHeight="1">
+          <t xml:space="preserve">traceback, исключение, try, except, finally, точка останова</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="60" customHeight="1">
       <c r="A22" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">22</t>
@@ -675,12 +675,12 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Разбор темы «Базовые алгоритмы сортировки и поиска»: ключевые понятия, примеры и практические ситуации.</t>
+          <t xml:space="preserve">Сравните пузырьковую сортировку, сортировку выбором и линейный поиск с бинарным по числу сравнений и условиям применимости.</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Базовые алгоритмы сортировки и поиска</t>
+          <t xml:space="preserve">обмен, проход по массиву, бинарный поиск, число сравнений, отсортированный массив, сложность</t>
         </is>
       </c>
     </row>
@@ -705,12 +705,12 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Совмещённая практическая работа: Множества: базовые задачи; Функции: базовые задачи.</t>
+          <t xml:space="preserve">Собираете функции для работы с наборами: объединение, пересечение, разность, и оформляете их как модуль с проверочными вызовами.</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Множества: базовые задачи, Функции: базовые задачи</t>
+          <t xml:space="preserve">объединение, пересечение, разность, аргумент функции, проверочный вызов</t>
         </is>
       </c>
     </row>
@@ -735,12 +735,12 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Совмещённая практическая работа: Рекурсия: базовые задачи; Модули: базовые задачи.</t>
+          <t xml:space="preserve">Пишете рекурсивные функции с базовым случаем и выносите их в отдельный модуль, который импортирует основной скрипт.</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Рекурсия: базовые задачи, Модули: базовые задачи</t>
+          <t xml:space="preserve">базовый случай, рекурсивный вызов, глубина рекурсии, import, пакет</t>
         </is>
       </c>
     </row>
@@ -765,12 +765,12 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Совмещённая практическая работа: Файлы: базовые задачи; Исключения: базовые задачи.</t>
+          <t xml:space="preserve">Строите программу, которая читает файл, перехватывает ошибки формата и записывает журнал обработки, и сдаёте её с набором тестовых файлов.</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Файлы: базовые задачи, Исключения: базовые задачи</t>
+          <t xml:space="preserve">FileNotFoundError, ValueError, журнал, разбор строки, кодировка</t>
         </is>
       </c>
     </row>
@@ -795,12 +795,12 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Совмещённая практическая работа: Сортировка: базовые задачи; Поиск: базовые задачи.</t>
+          <t xml:space="preserve">Реализуете сортировку и поиск на реальных наборах, замеряете число сравнений и сравниваете результат со встроенной функцией sorted.</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Сортировка: базовые задачи, Поиск: базовые задачи</t>
+          <t xml:space="preserve">устойчивость, sorted, ключ сортировки, линейный поиск, счётчик сравнений</t>
         </is>
       </c>
     </row>
@@ -825,12 +825,12 @@
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Совмещённая практическая работа: Двумерные массивы: базовые задачи; Алгоритмы на графах: базовые задачи.</t>
+          <t xml:space="preserve">Обрабатываете таблицу как вложенный список и обходите граф в ширину, сдавая программу с выводом пути и матрицы смежности.</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Двумерные массивы: базовые задачи, Алгоритмы на графах: базовые задачи</t>
+          <t xml:space="preserve">вложенный список, матрица смежности, обход в ширину, очередь, путь</t>
         </is>
       </c>
     </row>
@@ -855,12 +855,12 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Совмещённая практическая работа: Динамическое программирование: базовые задачи; Жадные алгоритмы: базовые задачи.</t>
+          <t xml:space="preserve">Решаете задачи, где жадный выбор не всегда верен, и сравниваете его с таблицей динамического программирования на одних данных.</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Динамическое программирование: базовые задачи, Жадные алгоритмы: базовые задачи</t>
+          <t xml:space="preserve">подзадача, таблица значений, жадный выбор, контрпример, оптимальность</t>
         </is>
       </c>
     </row>
@@ -885,12 +885,12 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Совмещённая практическая работа: Битовые операции: базовые задачи; Регулярные выражения: базовые задачи.</t>
+          <t xml:space="preserve">Работаете с двоичным представлением числа и разбираете строки шаблоном: маски, сдвиги и поиск по регулярному выражению.</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Битовые операции: базовые задачи, Регулярные выражения: базовые задачи</t>
+          <t xml:space="preserve">битовая маска, сдвиг, xor, шаблон, группа, re</t>
         </is>
       </c>
     </row>
@@ -915,12 +915,12 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Совмещённая практическая работа: Генераторы: базовые задачи; Декораторы: базовые задачи.</t>
+          <t xml:space="preserve">Пишете генератор, который отдаёт значения по одному, и оборачиваете функцию декоратором для замера времени и логирования.</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Генераторы: базовые задачи, Декораторы: базовые задачи</t>
+          <t xml:space="preserve">yield, итератор, ленивое вычисление, замыкание, обёртка, functools</t>
         </is>
       </c>
     </row>
@@ -945,12 +945,12 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Совмещённая практическая работа: ООП: базовые задачи; Наследование: базовые задачи.</t>
+          <t xml:space="preserve">Описываете предметную область классами с полями и методами и выносите общее поведение в базовый класс, сдавая модель из трёх классов.</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">ООП: базовые задачи, Наследование: базовые задачи</t>
+          <t xml:space="preserve">класс, экземпляр, метод, иерархия классов, переопределение, super</t>
         </is>
       </c>
     </row>
@@ -975,12 +975,12 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Совмещённая практическая работа: Тестирование: базовые задачи; Отладка: базовые задачи.</t>
+          <t xml:space="preserve">Пишете проверки для своих функций и находите ошибку в чужом коде по трассировке, сдавая набор тестов и отчёт о найденном дефекте.</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Тестирование: базовые задачи, Отладка: базовые задачи</t>
+          <t xml:space="preserve">assert, тестовый набор, граничное значение, точка останова, дефект</t>
         </is>
       </c>
     </row>
@@ -1005,12 +1005,12 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Совмещённая практическая работа: Работа с JSON: базовые задачи; Работа с CSV: базовые задачи.</t>
+          <t xml:space="preserve">Читаете и записываете обменные форматы: разбираете JSON в словарь и таблицу CSV в список строк, сдавая конвертер между форматами.</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Работа с JSON: базовые задачи, Работа с CSV: базовые задачи</t>
+          <t xml:space="preserve">json.load, сериализация, разделитель, заголовок, DictReader</t>
         </is>
       </c>
     </row>
@@ -1035,12 +1035,12 @@
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Совмещённая практическая работа: Мини-проект: базовые задачи; Итоговая работа: базовые задачи.</t>
+          <t xml:space="preserve">Собираете небольшую программу из готовых функций: ввод, обработка, сохранение отчёта, и защищаете её по чек-листу требований.</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Мини-проект: базовые задачи, Итоговая работа: базовые задачи</t>
+          <t xml:space="preserve">структура проекта, главная функция, обработка ввода, отчёт, защита работы</t>
         </is>
       </c>
     </row>
@@ -1065,12 +1065,12 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Совмещённая практическая работа: Ввод и вывод: прикладные задачи; Арифметические операции: прикладные задачи.</t>
+          <t xml:space="preserve">Решаете расчётные задачи с реальными данными: стоимость, скидка, перевод единиц, и сдаёте скрипт с проверкой на крайних значениях.</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ввод и вывод: прикладные задачи, Арифметические операции: прикладные задачи</t>
+          <t xml:space="preserve">формула, округление, единицы измерения, наценка, проверка расчёта</t>
         </is>
       </c>
     </row>
@@ -1095,12 +1095,12 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Совмещённая практическая работа: Разветвления: прикладные задачи; Циклы for: прикладные задачи.</t>
+          <t xml:space="preserve">Строите программу с выбором тарифа и накоплением итога по диапазону, сдавая её с таблицей результатов по нескольким входам.</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Разветвления: прикладные задачи, Циклы for: прикладные задачи</t>
+          <t xml:space="preserve">тариф, диапазон, накопитель, шаг цикла, таблица результатов</t>
         </is>
       </c>
     </row>
@@ -1125,12 +1125,12 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Совмещённая практическая работа: Циклы while: прикладные задачи; Вложенные циклы: прикладные задачи.</t>
+          <t xml:space="preserve">Моделируете процесс с условием остановки и строите сетку значений вложенным циклом, сдавая программу с журналом шагов.</t>
         </is>
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Циклы while: прикладные задачи, Вложенные циклы: прикладные задачи</t>
+          <t xml:space="preserve">условие остановки, моделирование, сетка значений, журнал шагов, итерация</t>
         </is>
       </c>
     </row>
@@ -1155,12 +1155,12 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Совмещённая практическая работа: Строки: прикладные задачи; Списки: прикладные задачи.</t>
+          <t xml:space="preserve">Разбираете текстовый отчёт: выделяете поля, считаете показатели по строкам и собираете сводку в список, готовый к выводу.</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Строки: прикладные задачи, Списки: прикладные задачи</t>
+          <t xml:space="preserve">разделитель, поле отчёта, сводка, среднее, форматирование вывода</t>
         </is>
       </c>
     </row>
@@ -1185,12 +1185,12 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Совмещённая практическая работа: Кортежи: прикладные задачи; Словари: прикладные задачи.</t>
+          <t xml:space="preserve">Храните справочник записей в словаре и используете кортеж как составной ключ, сдавая программу поиска и обновления записей.</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Кортежи: прикладные задачи, Словари: прикладные задачи</t>
+          <t xml:space="preserve">составной ключ, справочник, поиск записи, сортировка ключей, обновление</t>
         </is>
       </c>
     </row>
@@ -1215,12 +1215,12 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Совмещённая практическая работа: Множества: прикладные задачи; Функции: прикладные задачи.</t>
+          <t xml:space="preserve">Сравниваете два набора данных через множества и оформляете проверку как функцию, которую вызывают из основного сценария.</t>
         </is>
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Множества: прикладные задачи, Функции: прикладные задачи</t>
+          <t xml:space="preserve">разность множеств, пересечение, симметричная разность, возврат значения, повторный вызов</t>
         </is>
       </c>
     </row>
@@ -1245,12 +1245,12 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Совмещённая практическая работа: Рекурсия: прикладные задачи; Модули: прикладные задачи.</t>
+          <t xml:space="preserve">Реализуете обход вложенной структуры рекурсией и разносите код по двум модулям с общим пакетом, сдавая рабочую сборку.</t>
         </is>
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Рекурсия: прикладные задачи, Модули: прикладные задачи</t>
+          <t xml:space="preserve">вложенная структура, рекурсивный обход, пакет, относительный импорт, точка входа</t>
         </is>
       </c>
     </row>
@@ -1275,12 +1275,12 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Совмещённая практическая работа: Файлы: прикладные задачи; Исключения: прикладные задачи.</t>
+          <t xml:space="preserve">Строите обработчик журнала: читает файл построчно, пропускает битые строки с записью в отчёт и сохраняет очищенные данные.</t>
         </is>
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Файлы: прикладные задачи, Исключения: прикладные задачи</t>
+          <t xml:space="preserve">построчное чтение, битая строка, отчёт об ошибках, очистка данных, дозапись</t>
         </is>
       </c>
     </row>
@@ -1305,12 +1305,12 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Совмещённая практическая работа: Сортировка: прикладные задачи; Поиск: прикладные задачи.</t>
+          <t xml:space="preserve">Сортируете каталог по нескольким ключам и ищете записи по частичному совпадению, сдавая программу с замерами времени.</t>
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Сортировка: прикладные задачи, Поиск: прикладные задачи</t>
+          <t xml:space="preserve">составной ключ, частичное совпадение, time, индекс, бинарный поиск</t>
         </is>
       </c>
     </row>
@@ -1335,12 +1335,12 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Совмещённая практическая работа: Двумерные массивы: прикладные задачи; Алгоритмы на графах: прикладные задачи.</t>
+          <t xml:space="preserve">Строите матрицу расстояний по карте дорог и находите кратчайший путь обходом графа, сдавая программу с картой и маршрутом.</t>
         </is>
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Двумерные массивы: прикладные задачи, Алгоритмы на графах: прикладные задачи</t>
+          <t xml:space="preserve">матрица смежности, кратчайший путь, обход в ширину, маршрут, вес ребра</t>
         </is>
       </c>
     </row>
@@ -1365,12 +1365,12 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Совмещённая практическая работа: Динамическое программирование: прикладные задачи; Жадные алгоритмы: прикладные задачи.</t>
+          <t xml:space="preserve">Решаете задачу о размене и задачу о расписании двумя подходами, сравниваете ответы и объясняете расхождение в отчёте.</t>
         </is>
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Динамическое программирование: прикладные задачи, Жадные алгоритмы: прикладные задачи</t>
+          <t xml:space="preserve">размен, расписание, таблица решений, жадное правило, контрпример</t>
         </is>
       </c>
     </row>
@@ -1395,12 +1395,12 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Совмещённая практическая работа: Битовые операции: прикладные задачи; Регулярные выражения: прикладные задачи.</t>
+          <t xml:space="preserve">Кодируете набор флагов в одном числе и проверяете формат данных шаблоном, сдавая программу разбора и валидации строк.</t>
         </is>
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Битовые операции: прикладные задачи, Регулярные выражения: прикладные задачи</t>
+          <t xml:space="preserve">флаг, маска, сдвиг влево, валидация, именованная группа, re.fullmatch</t>
         </is>
       </c>
     </row>
@@ -1425,12 +1425,12 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Совмещённая практическая работа: Генераторы: прикладные задачи; Декораторы: прикладные задачи.</t>
+          <t xml:space="preserve">Обрабатываете поток записей генератором и добавляете к функциям замер времени, не меняя их код, сдавая программу с отчётом.</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Генераторы: прикладные задачи, Декораторы: прикладные задачи</t>
+          <t xml:space="preserve">поток данных, yield, замыкание, обёртка, время вызова, лог</t>
         </is>
       </c>
     </row>
@@ -1455,12 +1455,12 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Совмещённая практическая работа: ООП: прикладные задачи; Наследование: прикладные задачи.</t>
+          <t xml:space="preserve">Проектируете иерархию классов для учёта техники и проверяете её на наборе объектов, сдавая диаграмму и работающий код.</t>
         </is>
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">ООП: прикладные задачи, Наследование: прикладные задачи</t>
+          <t xml:space="preserve">базовый класс, наследник, полиморфизм, переопределение, иерархия</t>
         </is>
       </c>
     </row>
@@ -1485,12 +1485,12 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Совмещённая практическая работа: Тестирование: прикладные задачи; Отладка: прикладные задачи.</t>
+          <t xml:space="preserve">Покрываете готовый модуль проверками и устраняете найденный дефект, сдавая набор тестов и описание исправления.</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Тестирование: прикладные задачи, Отладка: прикладные задачи</t>
+          <t xml:space="preserve">покрытие ветвей, падающий тест, регрессия, assert, исправление</t>
         </is>
       </c>
     </row>
@@ -1515,12 +1515,12 @@
       </c>
       <c r="E50" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Совмещённая практическая работа: Работа с JSON: прикладные задачи; Работа с CSV: прикладные задачи.</t>
+          <t xml:space="preserve">Переносите данные между JSON и CSV без потери полей, сдавая конвертер, который проверен на файле с вложенными записями.</t>
         </is>
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Работа с JSON: прикладные задачи, Работа с CSV: прикладные задачи</t>
+          <t xml:space="preserve">вложенный объект, плоская таблица, экранирование, обратное преобразование, кодировка</t>
         </is>
       </c>
     </row>
@@ -1545,12 +1545,12 @@
       </c>
       <c r="E51" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Совмещённая практическая работа: Мини-проект: прикладные задачи; Итоговая работа: прикладные задачи.</t>
+          <t xml:space="preserve">Собираете приложение для учёта заявок с хранением в файле и защищаете его по требованиям к интерфейсу и обработке ошибок.</t>
         </is>
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Мини-проект: прикладные задачи, Итоговая работа: прикладные задачи</t>
+          <t xml:space="preserve">заявка, хранение, структура модулей, сценарий пользователя, защита</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Polish quizzes, plans, practices and templates
Quizzes now mix question types; Excel plans show academic hours; the landing describes the materials and lists the toolkit. Practices put all work under Ход работы, keep only evidence screenshots, drop self-check answers into a non-copyable question list, and code blocks carry language labels. Report templates gain a Ход работы section and lose answer fields and header screenshots; README is updated.
</commit_message>
<xml_diff>
--- a/courses/2/algorithms/dist/Учебный_план_Основы_алгоритмизации_и_программирования.xlsx
+++ b/courses/2/algorithms/dist/Учебный_план_Основы_алгоритмизации_и_программирования.xlsx
@@ -160,7 +160,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Минуты</t>
+          <t xml:space="preserve">Часы</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -191,7 +191,7 @@
         </is>
       </c>
       <c r="D6" s="6">
-        <v>90</v>
+        <v>2</v>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
@@ -221,7 +221,7 @@
         </is>
       </c>
       <c r="D7" s="6">
-        <v>90</v>
+        <v>2</v>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
@@ -251,7 +251,7 @@
         </is>
       </c>
       <c r="D8" s="6">
-        <v>180</v>
+        <v>4</v>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
@@ -281,7 +281,7 @@
         </is>
       </c>
       <c r="D9" s="6">
-        <v>90</v>
+        <v>2</v>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
@@ -311,7 +311,7 @@
         </is>
       </c>
       <c r="D10" s="6">
-        <v>90</v>
+        <v>2</v>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
@@ -341,7 +341,7 @@
         </is>
       </c>
       <c r="D11" s="6">
-        <v>180</v>
+        <v>4</v>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
@@ -371,7 +371,7 @@
         </is>
       </c>
       <c r="D12" s="6">
-        <v>90</v>
+        <v>2</v>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
@@ -401,7 +401,7 @@
         </is>
       </c>
       <c r="D13" s="6">
-        <v>90</v>
+        <v>2</v>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
@@ -431,7 +431,7 @@
         </is>
       </c>
       <c r="D14" s="6">
-        <v>180</v>
+        <v>4</v>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
@@ -461,7 +461,7 @@
         </is>
       </c>
       <c r="D15" s="6">
-        <v>90</v>
+        <v>2</v>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
@@ -491,7 +491,7 @@
         </is>
       </c>
       <c r="D16" s="6">
-        <v>90</v>
+        <v>2</v>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
@@ -521,7 +521,7 @@
         </is>
       </c>
       <c r="D17" s="6">
-        <v>180</v>
+        <v>4</v>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
@@ -551,7 +551,7 @@
         </is>
       </c>
       <c r="D18" s="6">
-        <v>90</v>
+        <v>2</v>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
@@ -581,7 +581,7 @@
         </is>
       </c>
       <c r="D19" s="6">
-        <v>90</v>
+        <v>2</v>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
@@ -611,7 +611,7 @@
         </is>
       </c>
       <c r="D20" s="6">
-        <v>180</v>
+        <v>4</v>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="D21" s="6">
-        <v>90</v>
+        <v>2</v>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
@@ -671,7 +671,7 @@
         </is>
       </c>
       <c r="D22" s="6">
-        <v>90</v>
+        <v>2</v>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
@@ -701,7 +701,7 @@
         </is>
       </c>
       <c r="D23" s="6">
-        <v>180</v>
+        <v>4</v>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
@@ -731,7 +731,7 @@
         </is>
       </c>
       <c r="D24" s="6">
-        <v>180</v>
+        <v>4</v>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
@@ -761,7 +761,7 @@
         </is>
       </c>
       <c r="D25" s="6">
-        <v>180</v>
+        <v>4</v>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
@@ -791,7 +791,7 @@
         </is>
       </c>
       <c r="D26" s="6">
-        <v>180</v>
+        <v>4</v>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
@@ -821,7 +821,7 @@
         </is>
       </c>
       <c r="D27" s="6">
-        <v>180</v>
+        <v>4</v>
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
@@ -851,7 +851,7 @@
         </is>
       </c>
       <c r="D28" s="6">
-        <v>180</v>
+        <v>4</v>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
@@ -881,7 +881,7 @@
         </is>
       </c>
       <c r="D29" s="6">
-        <v>180</v>
+        <v>4</v>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="D30" s="6">
-        <v>180</v>
+        <v>4</v>
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
@@ -941,7 +941,7 @@
         </is>
       </c>
       <c r="D31" s="6">
-        <v>180</v>
+        <v>4</v>
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
@@ -971,7 +971,7 @@
         </is>
       </c>
       <c r="D32" s="6">
-        <v>180</v>
+        <v>4</v>
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
@@ -1001,7 +1001,7 @@
         </is>
       </c>
       <c r="D33" s="6">
-        <v>180</v>
+        <v>4</v>
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
@@ -1031,7 +1031,7 @@
         </is>
       </c>
       <c r="D34" s="6">
-        <v>180</v>
+        <v>4</v>
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
@@ -1061,7 +1061,7 @@
         </is>
       </c>
       <c r="D35" s="6">
-        <v>180</v>
+        <v>4</v>
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
@@ -1091,7 +1091,7 @@
         </is>
       </c>
       <c r="D36" s="6">
-        <v>180</v>
+        <v>4</v>
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
@@ -1121,7 +1121,7 @@
         </is>
       </c>
       <c r="D37" s="6">
-        <v>180</v>
+        <v>4</v>
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
@@ -1151,7 +1151,7 @@
         </is>
       </c>
       <c r="D38" s="6">
-        <v>180</v>
+        <v>4</v>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
@@ -1181,7 +1181,7 @@
         </is>
       </c>
       <c r="D39" s="6">
-        <v>180</v>
+        <v>4</v>
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
@@ -1211,7 +1211,7 @@
         </is>
       </c>
       <c r="D40" s="6">
-        <v>180</v>
+        <v>4</v>
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="D41" s="6">
-        <v>180</v>
+        <v>4</v>
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
@@ -1271,7 +1271,7 @@
         </is>
       </c>
       <c r="D42" s="6">
-        <v>180</v>
+        <v>4</v>
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
@@ -1301,7 +1301,7 @@
         </is>
       </c>
       <c r="D43" s="6">
-        <v>180</v>
+        <v>4</v>
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
@@ -1331,7 +1331,7 @@
         </is>
       </c>
       <c r="D44" s="6">
-        <v>180</v>
+        <v>4</v>
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
@@ -1361,7 +1361,7 @@
         </is>
       </c>
       <c r="D45" s="6">
-        <v>180</v>
+        <v>4</v>
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
@@ -1391,7 +1391,7 @@
         </is>
       </c>
       <c r="D46" s="6">
-        <v>180</v>
+        <v>4</v>
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
@@ -1421,7 +1421,7 @@
         </is>
       </c>
       <c r="D47" s="6">
-        <v>180</v>
+        <v>4</v>
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
@@ -1451,7 +1451,7 @@
         </is>
       </c>
       <c r="D48" s="6">
-        <v>180</v>
+        <v>4</v>
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
@@ -1481,7 +1481,7 @@
         </is>
       </c>
       <c r="D49" s="6">
-        <v>180</v>
+        <v>4</v>
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
@@ -1511,7 +1511,7 @@
         </is>
       </c>
       <c r="D50" s="6">
-        <v>180</v>
+        <v>4</v>
       </c>
       <c r="E50" s="5" t="inlineStr">
         <is>
@@ -1541,7 +1541,7 @@
         </is>
       </c>
       <c r="D51" s="6">
-        <v>180</v>
+        <v>4</v>
       </c>
       <c r="E51" s="5" t="inlineStr">
         <is>
@@ -1571,7 +1571,7 @@
         </is>
       </c>
       <c r="D52" s="6">
-        <v>7200</v>
+        <v>160</v>
       </c>
       <c r="E52" s="6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add all IS implementation lessons and fix lecture-practice order
- write 38 lessons for MDK.06.01: 24 lectures and 14 practices
- reorder all planned courses so each practice follows the lecture that introduces its topic
- change specialty summary on the landing from courses to streams
- document the lecture-before-practice rule in AGENTS and the course skill
</commit_message>
<xml_diff>
--- a/courses/2/algorithms/dist/Учебный_план_Основы_алгоритмизации_и_программирования.xlsx
+++ b/courses/2/algorithms/dist/Учебный_план_Основы_алгоритмизации_и_программирования.xlsx
@@ -237,60 +237,60 @@
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">3-4</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика</t>
+          <t xml:space="preserve">Лекция</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 1. Ввод и вывод: базовые задачи; Арифметические операции: базовые задачи</t>
+          <t xml:space="preserve">Лекция 3. Переменные, типы и выражения</t>
         </is>
       </c>
       <c r="D8" s="6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Пишете в VS Code программы, которые читают числа через input и печатают результат арифметики, и сдаёте набор из пяти работающих скриптов с выводом.</t>
+          <t xml:space="preserve">Разберёте, как Python хранит значение в переменной, почему 0.1 + 0.2 даёт хвост и когда неявное приведение типов ломает расчёт.</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">input, int, float, f-строка, деление нацело, остаток</t>
+          <t xml:space="preserve">переменная, динамическая типизация, приведение типов, приоритет операций, округление</t>
         </is>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">5</t>
+          <t xml:space="preserve">4-5</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция</t>
+          <t xml:space="preserve">Практика</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция 3. Переменные, типы и выражения</t>
+          <t xml:space="preserve">Практика 1. Ввод и вывод: базовые задачи; Арифметические операции: базовые задачи</t>
         </is>
       </c>
       <c r="D9" s="6">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Разберёте, как Python хранит значение в переменной, почему 0.1 + 0.2 даёт хвост и когда неявное приведение типов ломает расчёт.</t>
+          <t xml:space="preserve">Пишете в VS Code программы, которые читают числа через input и печатают результат арифметики, и сдаёте набор из пяти работающих скриптов с выводом.</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">переменная, динамическая типизация, приведение типов, приоритет операций, округление</t>
+          <t xml:space="preserve">input, int, float, f-строка, деление нацело, остаток</t>
         </is>
       </c>
     </row>
@@ -327,120 +327,120 @@
     <row r="11" ht="45" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">7-8</t>
+          <t xml:space="preserve">7</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика</t>
+          <t xml:space="preserve">Лекция</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 2. Разветвления: базовые задачи; Циклы for: базовые задачи</t>
+          <t xml:space="preserve">Лекция 5. Циклы</t>
         </is>
       </c>
       <c r="D11" s="6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Решаете задачи на выбор варианта и перебор диапазона: программы с if, elif и for, проверенные на наборе входных значений.</t>
+          <t xml:space="preserve">Сравните for и while, разберёте, откуда берётся бесконечный цикл, и научитесь останавливать перебор через break и continue.</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">range, ветвление, счётчик, накопление суммы, тестовый набор</t>
+          <t xml:space="preserve">for, while, break, continue, счётчик итераций, условие выхода</t>
         </is>
       </c>
     </row>
     <row r="12" ht="45" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">9</t>
+          <t xml:space="preserve">8-9</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция</t>
+          <t xml:space="preserve">Практика</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция 5. Циклы</t>
+          <t xml:space="preserve">Практика 2. Разветвления: базовые задачи; Циклы for: базовые задачи</t>
         </is>
       </c>
       <c r="D12" s="6">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Сравните for и while, разберёте, откуда берётся бесконечный цикл, и научитесь останавливать перебор через break и continue.</t>
+          <t xml:space="preserve">Решаете задачи на выбор варианта и перебор диапазона: программы с if, elif и for, проверенные на наборе входных значений.</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">for, while, break, continue, счётчик итераций, условие выхода</t>
+          <t xml:space="preserve">range, ветвление, счётчик, накопление суммы, тестовый набор</t>
         </is>
       </c>
     </row>
     <row r="13" ht="45" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">10</t>
+          <t xml:space="preserve">10-11</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция</t>
+          <t xml:space="preserve">Практика</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция 6. Массивы и списки</t>
+          <t xml:space="preserve">Практика 3. Циклы while: базовые задачи; Вложенные циклы: базовые задачи</t>
         </is>
       </c>
       <c r="D13" s="6">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Разберёте, как список хранит элементы по индексам, что делает срез и почему вставка в середину дороже добавления в конец.</t>
+          <t xml:space="preserve">Пишете программы с while и вложенным перебором: таблицы, суммы рядов и поиск до условия, с проверкой числа итераций.</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">индекс, срез, append, вложенный список, длина списка</t>
+          <t xml:space="preserve">while True, вложенный цикл, внешний счётчик, таблица, валидация ввода</t>
         </is>
       </c>
     </row>
     <row r="14" ht="45" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">11-12</t>
+          <t xml:space="preserve">12</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика</t>
+          <t xml:space="preserve">Лекция</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 3. Циклы while: базовые задачи; Вложенные циклы: базовые задачи</t>
+          <t xml:space="preserve">Лекция 6. Массивы и списки</t>
         </is>
       </c>
       <c r="D14" s="6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Пишете программы с while и вложенным перебором: таблицы, суммы рядов и поиск до условия, с проверкой числа итераций.</t>
+          <t xml:space="preserve">Разберёте, как список хранит элементы по индексам, что делает срез и почему вставка в середину дороже добавления в конец.</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">while True, вложенный цикл, внешний счётчик, таблица, валидация ввода</t>
+          <t xml:space="preserve">индекс, срез, append, вложенный список, длина списка</t>
         </is>
       </c>
     </row>
@@ -477,60 +477,60 @@
     <row r="16" ht="45" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">14</t>
+          <t xml:space="preserve">14-15</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция</t>
+          <t xml:space="preserve">Практика</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция 8. Функции и модули</t>
+          <t xml:space="preserve">Практика 4. Строки: базовые задачи; Списки: базовые задачи</t>
         </is>
       </c>
       <c r="D16" s="6">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Разберёте, зачем выносить код в функцию, как передаются аргументы и как собрать свои функции в модуль, который импортируют другие файлы.</t>
+          <t xml:space="preserve">Обрабатываете текст и наборы данных: подсчёт слов, очистка строк, сортировка списка, и сдаёте скрипты с разбором сложных случаев.</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">def, return, параметр, область видимости, import, докстрока</t>
+          <t xml:space="preserve">частота, фильтрация, сортировка, пустой ввод, нормализация</t>
         </is>
       </c>
     </row>
     <row r="17" ht="45" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">15-16</t>
+          <t xml:space="preserve">16</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика</t>
+          <t xml:space="preserve">Лекция</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 4. Строки: базовые задачи; Списки: базовые задачи</t>
+          <t xml:space="preserve">Лекция 8. Функции и модули</t>
         </is>
       </c>
       <c r="D17" s="6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Обрабатываете текст и наборы данных: подсчёт слов, очистка строк, сортировка списка, и сдаёте скрипты с разбором сложных случаев.</t>
+          <t xml:space="preserve">Разберёте, зачем выносить код в функцию, как передаются аргументы и как собрать свои функции в модуль, который импортируют другие файлы.</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">частота, фильтрация, сортировка, пустой ввод, нормализация</t>
+          <t xml:space="preserve">def, return, параметр, область видимости, import, докстрока</t>
         </is>
       </c>
     </row>
@@ -567,37 +567,37 @@
     <row r="19" ht="45" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">18</t>
+          <t xml:space="preserve">18-19</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция</t>
+          <t xml:space="preserve">Практика</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция 10. Файлы и обработка данных</t>
+          <t xml:space="preserve">Практика 5. Кортежи: базовые задачи; Словари: базовые задачи</t>
         </is>
       </c>
       <c r="D19" s="6">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Научитесь читать и записывать текстовые файлы через with, не теряя данные при ошибке, и обрабатывать строки файла построчно.</t>
+          <t xml:space="preserve">Работаете с неизменяемыми наборами и справочниками: кортеж как ключ, словарь как база записей, и сдаёте программу с отчётом по данным.</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">open, with, режим доступа, кодировка, чтение строк, буфер</t>
+          <t xml:space="preserve">неизменяемый набор, распаковка, вложенный словарь, get, обновление записи</t>
         </is>
       </c>
     </row>
     <row r="20" ht="45" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">19-20</t>
+          <t xml:space="preserve">20-21</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
@@ -607,7 +607,7 @@
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 5. Кортежи: базовые задачи; Словари: базовые задачи</t>
+          <t xml:space="preserve">Практика 6. Множества: базовые задачи; Функции: базовые задачи</t>
         </is>
       </c>
       <c r="D20" s="6">
@@ -615,19 +615,19 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Работаете с неизменяемыми наборами и справочниками: кортеж как ключ, словарь как база записей, и сдаёте программу с отчётом по данным.</t>
+          <t xml:space="preserve">Собираете функции для работы с наборами: объединение, пересечение, разность, и оформляете их как модуль с проверочными вызовами.</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">неизменяемый набор, распаковка, вложенный словарь, get, обновление записи</t>
+          <t xml:space="preserve">объединение, пересечение, разность, аргумент функции, проверочный вызов</t>
         </is>
       </c>
     </row>
     <row r="21" ht="45" customHeight="1">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">21</t>
+          <t xml:space="preserve">22</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
@@ -637,7 +637,7 @@
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция 11. Ошибки, исключения и отладка</t>
+          <t xml:space="preserve">Лекция 10. Файлы и обработка данных</t>
         </is>
       </c>
       <c r="D21" s="6">
@@ -645,19 +645,19 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Разберёте три вида ошибок, научитесь читать трассировку Python и обрабатывать сбой через try, except и finally вместо падения программы.</t>
+          <t xml:space="preserve">Научитесь читать и записывать текстовые файлы через with, не теряя данные при ошибке, и обрабатывать строки файла построчно.</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">traceback, исключение, try, except, finally, точка останова</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="60" customHeight="1">
+          <t xml:space="preserve">open, with, режим доступа, кодировка, чтение строк, буфер</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="45" customHeight="1">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">22</t>
+          <t xml:space="preserve">23</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -667,7 +667,7 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция 12. Базовые алгоритмы сортировки и поиска</t>
+          <t xml:space="preserve">Лекция 11. Ошибки, исключения и отладка</t>
         </is>
       </c>
       <c r="D22" s="6">
@@ -675,42 +675,42 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">Разберёте три вида ошибок, научитесь читать трассировку Python и обрабатывать сбой через try, except и finally вместо падения программы.</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">traceback, исключение, try, except, finally, точка останова</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="60" customHeight="1">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">24</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Лекция</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Лекция 12. Базовые алгоритмы сортировки и поиска</t>
+        </is>
+      </c>
+      <c r="D23" s="6">
+        <v>2</v>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">Сравните пузырьковую сортировку, сортировку выбором и линейный поиск с бинарным по числу сравнений и условиям применимости.</t>
         </is>
       </c>
-      <c r="F22" s="5" t="inlineStr">
+      <c r="F23" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">обмен, проход по массиву, бинарный поиск, число сравнений, отсортированный массив, сложность</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="45" customHeight="1">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">23-24</t>
-        </is>
-      </c>
-      <c r="B23" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Практика</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Практика 6. Множества: базовые задачи; Функции: базовые задачи</t>
-        </is>
-      </c>
-      <c r="D23" s="6">
-        <v>4</v>
-      </c>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Собираете функции для работы с наборами: объединение, пересечение, разность, и оформляете их как модуль с проверочными вызовами.</t>
-        </is>
-      </c>
-      <c r="F23" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">объединение, пересечение, разность, аргумент функции, проверочный вызов</t>
         </is>
       </c>
     </row>

</xml_diff>